<commit_message>
mlflow baseline done, now just smaller optimizations for better score
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AALB\Desktop\mp\graph\graphxmaf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C4ACC2-B0B4-4BE7-9B20-0CB32EA1F032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC88BE38-169A-4920-BDC8-76D5642B8C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graph" sheetId="1" r:id="rId1"/>
@@ -48220,7 +48220,7 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="80" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="142" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="56" customWidth="1"/>

</xml_diff>

<commit_message>
results + runs + extra
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AALB\Desktop\mp\graph\graphxmaf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC88BE38-169A-4920-BDC8-76D5642B8C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7762B742-1584-47FA-AD0A-07563730041B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3255" yWindow="5640" windowWidth="28800" windowHeight="15345" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graph" sheetId="1" r:id="rId1"/>
@@ -54186,7 +54186,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -55232,6 +55232,12 @@
         <v>1770</v>
       </c>
     </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J32">
+        <f>AVERAGE(J23:J26)</f>
+        <v>3.915</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>